<commit_message>
Optimize Routing: Factor in 50km discount pre-solving and enforce strict 3-site capacity
</commit_message>
<xml_diff>
--- a/Backend_Portal/uploads/test_output.xlsx
+++ b/Backend_Portal/uploads/test_output.xlsx
@@ -463,14 +463,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>I-RJ-KOTA-ENB-0049</t>
+          <t>I-RJ-GGPC-ENB-I011</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>25.14866</v>
+        <v>26.5470180555556</v>
       </c>
       <c r="C2" t="n">
-        <v>75.86027</v>
+        <v>76.8586008333333</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -483,20 +483,20 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>223.69</v>
+        <v>127.99</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>I-RJ-KOTA-ENB-0551</t>
+          <t>I-RJ-BUND-ENB-9031</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>25.2006977777778</v>
+        <v>25.4284158333333</v>
       </c>
       <c r="C3" t="n">
-        <v>75.85985805555551</v>
+        <v>75.7121338888889</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -505,24 +505,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>7.46</v>
+        <v>192.85</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>I-RJ-INDA-ENB-9031</t>
+          <t>I-RJ-BUND-ENB-9045</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>25.7305877777778</v>
+        <v>25.3781877777778</v>
       </c>
       <c r="C4" t="n">
-        <v>76.2218413888889</v>
+        <v>75.6110516666667</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -531,24 +531,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>83.54000000000001</v>
+        <v>17.91</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>I-RJ-RGMD-ENB-V002</t>
+          <t>I-RJ-BUND-ENB-9079</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>24.644986</v>
+        <v>25.4104888888889</v>
       </c>
       <c r="C5" t="n">
-        <v>75.941755</v>
+        <v>75.59469222222221</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -557,24 +557,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>294.62</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>I-RJ-SKET-ENB-9001</t>
+          <t>I-RJ-KOTA-ENB-0049</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>24.6421075</v>
+        <v>25.14866</v>
       </c>
       <c r="C6" t="n">
-        <v>76.0404627777778</v>
+        <v>75.86027</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -583,24 +583,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>11.3</v>
+        <v>223.69</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>I-RJ-SKET-ENB-6000</t>
+          <t>I-RJ-KOTA-ENB-0551</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>24.6503216666667</v>
+        <v>25.2006977777778</v>
       </c>
       <c r="C7" t="n">
-        <v>76.0430563888889</v>
+        <v>75.85985805555551</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -609,24 +609,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1.02</v>
+        <v>7.46</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>I-RJ-CHEH-ENB-9001</t>
+          <t>I-RJ-INDA-ENB-9031</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24.76928</v>
+        <v>25.7305877777778</v>
       </c>
       <c r="C8" t="n">
-        <v>75.88552</v>
+        <v>76.2218413888889</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -635,24 +635,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>289.34</v>
+        <v>83.53</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>I-RJ-MDKK-ENB-9001</t>
+          <t>I-RJ-DIRS-ENB-9024</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>24.71955</v>
+        <v>25.1538969444444</v>
       </c>
       <c r="C9" t="n">
-        <v>75.95354</v>
+        <v>76.1693158333333</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -661,24 +661,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>9.859999999999999</v>
+        <v>220.05</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>I-RJ-UDPU-ENB-9001</t>
+          <t>I-RJ-KOTA-ENB-0542</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24.7257102777778</v>
+        <v>25.1800027777778</v>
       </c>
       <c r="C10" t="n">
-        <v>75.9753980555556</v>
+        <v>75.8829472222222</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -687,24 +687,24 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>3.41</v>
+        <v>31.45</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>I-RJ-DIRS-ENB-9024</t>
+          <t>I-RJ-KOTA-ENB-0314</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>25.1538969444444</v>
+        <v>25.2037725</v>
       </c>
       <c r="C11" t="n">
-        <v>76.1693158333333</v>
+        <v>75.8439569444444</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -713,24 +713,24 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>220.05</v>
+        <v>5.83</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>I-RJ-KOTA-ENB-0542</t>
+          <t>I-RJ-RGMD-ENB-V002</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>25.1800027777778</v>
+        <v>24.644986</v>
       </c>
       <c r="C12" t="n">
-        <v>75.8829472222222</v>
+        <v>75.941755</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -739,24 +739,24 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>31.46</v>
+        <v>294.62</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>I-RJ-KOTA-ENB-0314</t>
+          <t>I-RJ-SKET-ENB-9001</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>25.2037725</v>
+        <v>24.6421075</v>
       </c>
       <c r="C13" t="n">
-        <v>75.8439569444444</v>
+        <v>76.0404627777778</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -765,24 +765,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>5.83</v>
+        <v>11.3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>I-RJ-BUND-ENB-9031</t>
+          <t>I-RJ-SKET-ENB-6000</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>25.4284158333333</v>
+        <v>24.6503216666667</v>
       </c>
       <c r="C14" t="n">
-        <v>75.7121338888889</v>
+        <v>76.0430563888889</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -791,24 +791,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>192.85</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>I-RJ-BUND-ENB-9045</t>
+          <t>I-RJ-CHEH-ENB-9001</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>25.3781877777778</v>
+        <v>24.76928</v>
       </c>
       <c r="C15" t="n">
-        <v>75.6110516666667</v>
+        <v>75.88552</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -817,24 +817,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>17.91</v>
+        <v>289.34</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>I-RJ-BUND-ENB-9079</t>
+          <t>I-RJ-MDKK-ENB-9001</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>25.4104888888889</v>
+        <v>24.71955</v>
       </c>
       <c r="C16" t="n">
-        <v>75.59469222222221</v>
+        <v>75.95354</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -843,24 +843,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.52</v>
+        <v>9.859999999999999</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>I-RJ-GGPC-ENB-I011</t>
+          <t>I-RJ-UDPU-ENB-9001</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>26.5470180555556</v>
+        <v>24.7257102777778</v>
       </c>
       <c r="C17" t="n">
-        <v>76.8586008333333</v>
+        <v>75.9753980555556</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -869,11 +869,11 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>127.99</v>
+        <v>3.41</v>
       </c>
     </row>
     <row r="18">

</xml_diff>